<commit_message>
Update project files and add SignUp page
</commit_message>
<xml_diff>
--- a/backend/tests/e2e-test-report.xlsx
+++ b/backend/tests/e2e-test-report.xlsx
@@ -445,13 +445,13 @@
         <v>PASS</v>
       </c>
       <c r="E2">
-        <v>1675</v>
+        <v>1543</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-06-12T09:32:30.672Z</v>
+        <v>2026-06-23T09:23:55.188Z</v>
       </c>
     </row>
     <row r="3">
@@ -468,13 +468,13 @@
         <v>PASS</v>
       </c>
       <c r="E3">
-        <v>601</v>
+        <v>817</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>2026-06-12T09:32:31.273Z</v>
+        <v>2026-06-23T09:23:56.006Z</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>PASS</v>
       </c>
       <c r="E4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F4" t="str">
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>2026-06-12T09:32:31.279Z</v>
+        <v>2026-06-23T09:23:56.018Z</v>
       </c>
     </row>
     <row r="5">
@@ -514,13 +514,13 @@
         <v>PASS</v>
       </c>
       <c r="E5">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F5" t="str">
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>2026-06-12T09:32:31.307Z</v>
+        <v>2026-06-23T09:23:56.043Z</v>
       </c>
     </row>
     <row r="6">
@@ -537,13 +537,13 @@
         <v>PASS</v>
       </c>
       <c r="E6">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F6" t="str">
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>2026-06-12T09:32:31.322Z</v>
+        <v>2026-06-23T09:23:56.061Z</v>
       </c>
     </row>
     <row r="7">
@@ -560,13 +560,13 @@
         <v>PASS</v>
       </c>
       <c r="E7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" t="str">
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>2026-06-12T09:32:31.331Z</v>
+        <v>2026-06-23T09:23:56.071Z</v>
       </c>
     </row>
     <row r="8">
@@ -583,13 +583,13 @@
         <v>PASS</v>
       </c>
       <c r="E8">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F8" t="str">
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>2026-06-12T09:32:31.342Z</v>
+        <v>2026-06-23T09:23:56.099Z</v>
       </c>
     </row>
     <row r="9">
@@ -606,13 +606,13 @@
         <v>PASS</v>
       </c>
       <c r="E9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" t="str">
         <v/>
       </c>
       <c r="G9" t="str">
-        <v>2026-06-12T09:32:31.352Z</v>
+        <v>2026-06-23T09:23:56.108Z</v>
       </c>
     </row>
     <row r="10">
@@ -629,13 +629,13 @@
         <v>PASS</v>
       </c>
       <c r="E10">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F10" t="str">
         <v/>
       </c>
       <c r="G10" t="str">
-        <v>2026-06-12T09:32:31.360Z</v>
+        <v>2026-06-23T09:23:56.118Z</v>
       </c>
     </row>
     <row r="11">
@@ -652,13 +652,13 @@
         <v>PASS</v>
       </c>
       <c r="E11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F11" t="str">
         <v/>
       </c>
       <c r="G11" t="str">
-        <v>2026-06-12T09:32:31.380Z</v>
+        <v>2026-06-23T09:23:56.145Z</v>
       </c>
     </row>
     <row r="12">
@@ -675,13 +675,13 @@
         <v>PASS</v>
       </c>
       <c r="E12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" t="str">
         <v/>
       </c>
       <c r="G12" t="str">
-        <v>2026-06-12T09:32:31.389Z</v>
+        <v>2026-06-23T09:23:56.153Z</v>
       </c>
     </row>
     <row r="13">
@@ -698,13 +698,13 @@
         <v>PASS</v>
       </c>
       <c r="E13">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="F13" t="str">
         <v/>
       </c>
       <c r="G13" t="str">
-        <v>2026-06-12T09:32:31.413Z</v>
+        <v>2026-06-23T09:23:56.160Z</v>
       </c>
     </row>
     <row r="14">
@@ -721,13 +721,13 @@
         <v>PASS</v>
       </c>
       <c r="E14">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F14" t="str">
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>2026-06-12T09:32:31.436Z</v>
+        <v>2026-06-23T09:23:56.184Z</v>
       </c>
     </row>
     <row r="15">
@@ -744,13 +744,13 @@
         <v>PASS</v>
       </c>
       <c r="E15">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F15" t="str">
         <v/>
       </c>
       <c r="G15" t="str">
-        <v>2026-06-12T09:32:31.445Z</v>
+        <v>2026-06-23T09:23:56.193Z</v>
       </c>
     </row>
     <row r="16">
@@ -767,13 +767,13 @@
         <v>PASS</v>
       </c>
       <c r="E16">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F16" t="str">
         <v/>
       </c>
       <c r="G16" t="str">
-        <v>2026-06-12T09:32:31.453Z</v>
+        <v>2026-06-23T09:23:56.208Z</v>
       </c>
     </row>
     <row r="17">
@@ -790,13 +790,13 @@
         <v>PASS</v>
       </c>
       <c r="E17">
-        <v>1273</v>
+        <v>1301</v>
       </c>
       <c r="F17" t="str">
         <v/>
       </c>
       <c r="G17" t="str">
-        <v>2026-06-12T09:32:32.727Z</v>
+        <v>2026-06-23T09:23:57.509Z</v>
       </c>
     </row>
     <row r="18">
@@ -813,13 +813,13 @@
         <v>PASS</v>
       </c>
       <c r="E18">
-        <v>1276</v>
+        <v>1290</v>
       </c>
       <c r="F18" t="str">
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>2026-06-12T09:32:34.003Z</v>
+        <v>2026-06-23T09:23:58.799Z</v>
       </c>
     </row>
     <row r="19">
@@ -836,13 +836,13 @@
         <v>PASS</v>
       </c>
       <c r="E19">
-        <v>1277</v>
+        <v>1316</v>
       </c>
       <c r="F19" t="str">
         <v/>
       </c>
       <c r="G19" t="str">
-        <v>2026-06-12T09:32:35.280Z</v>
+        <v>2026-06-23T09:24:00.115Z</v>
       </c>
     </row>
     <row r="20">
@@ -859,13 +859,13 @@
         <v>PASS</v>
       </c>
       <c r="E20">
-        <v>1308</v>
+        <v>1332</v>
       </c>
       <c r="F20" t="str">
         <v/>
       </c>
       <c r="G20" t="str">
-        <v>2026-06-12T09:32:36.588Z</v>
+        <v>2026-06-23T09:24:01.447Z</v>
       </c>
     </row>
     <row r="21">
@@ -882,13 +882,13 @@
         <v>PASS</v>
       </c>
       <c r="E21">
-        <v>1290</v>
+        <v>1327</v>
       </c>
       <c r="F21" t="str">
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>2026-06-12T09:32:37.879Z</v>
+        <v>2026-06-23T09:24:02.774Z</v>
       </c>
     </row>
     <row r="22">
@@ -905,13 +905,13 @@
         <v>PASS</v>
       </c>
       <c r="E22">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="F22" t="str">
         <v/>
       </c>
       <c r="G22" t="str">
-        <v>2026-06-12T09:32:39.186Z</v>
+        <v>2026-06-23T09:24:04.080Z</v>
       </c>
     </row>
     <row r="23">
@@ -928,13 +928,13 @@
         <v>PASS</v>
       </c>
       <c r="E23">
-        <v>1335</v>
+        <v>1322</v>
       </c>
       <c r="F23" t="str">
         <v/>
       </c>
       <c r="G23" t="str">
-        <v>2026-06-12T09:32:40.521Z</v>
+        <v>2026-06-23T09:24:05.402Z</v>
       </c>
     </row>
     <row r="24">
@@ -951,13 +951,13 @@
         <v>PASS</v>
       </c>
       <c r="E24">
-        <v>1307</v>
+        <v>1319</v>
       </c>
       <c r="F24" t="str">
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>2026-06-12T09:32:41.828Z</v>
+        <v>2026-06-23T09:24:06.721Z</v>
       </c>
     </row>
     <row r="25">
@@ -974,13 +974,13 @@
         <v>PASS</v>
       </c>
       <c r="E25">
-        <v>1296</v>
+        <v>1325</v>
       </c>
       <c r="F25" t="str">
         <v/>
       </c>
       <c r="G25" t="str">
-        <v>2026-06-12T09:32:43.124Z</v>
+        <v>2026-06-23T09:24:08.047Z</v>
       </c>
     </row>
     <row r="26">
@@ -997,13 +997,13 @@
         <v>PASS</v>
       </c>
       <c r="E26">
-        <v>1299</v>
+        <v>1306</v>
       </c>
       <c r="F26" t="str">
         <v/>
       </c>
       <c r="G26" t="str">
-        <v>2026-06-12T09:32:44.423Z</v>
+        <v>2026-06-23T09:24:09.353Z</v>
       </c>
     </row>
     <row r="27">
@@ -1020,13 +1020,13 @@
         <v>PASS</v>
       </c>
       <c r="E27">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="F27" t="str">
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>2026-06-12T09:32:44.730Z</v>
+        <v>2026-06-23T09:24:09.683Z</v>
       </c>
     </row>
     <row r="28">
@@ -1043,13 +1043,13 @@
         <v>PASS</v>
       </c>
       <c r="E28">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F28" t="str">
         <v/>
       </c>
       <c r="G28" t="str">
-        <v>2026-06-12T09:32:44.736Z</v>
+        <v>2026-06-23T09:24:09.686Z</v>
       </c>
     </row>
     <row r="29">
@@ -1066,13 +1066,13 @@
         <v>PASS</v>
       </c>
       <c r="E29">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="F29" t="str">
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>2026-06-12T09:32:44.770Z</v>
+        <v>2026-06-23T09:24:09.696Z</v>
       </c>
     </row>
     <row r="30">
@@ -1089,13 +1089,13 @@
         <v>PASS</v>
       </c>
       <c r="E30">
-        <v>1328</v>
+        <v>1322</v>
       </c>
       <c r="F30" t="str">
         <v/>
       </c>
       <c r="G30" t="str">
-        <v>2026-06-12T09:32:46.098Z</v>
+        <v>2026-06-23T09:24:11.018Z</v>
       </c>
     </row>
     <row r="31">
@@ -1112,13 +1112,13 @@
         <v>PASS</v>
       </c>
       <c r="E31">
-        <v>1310</v>
+        <v>1281</v>
       </c>
       <c r="F31" t="str">
         <v/>
       </c>
       <c r="G31" t="str">
-        <v>2026-06-12T09:32:47.409Z</v>
+        <v>2026-06-23T09:24:12.299Z</v>
       </c>
     </row>
     <row r="32">
@@ -1135,13 +1135,13 @@
         <v>PASS</v>
       </c>
       <c r="E32">
-        <v>593</v>
+        <v>608</v>
       </c>
       <c r="F32" t="str">
         <v/>
       </c>
       <c r="G32" t="str">
-        <v>2026-06-12T09:32:48.002Z</v>
+        <v>2026-06-23T09:24:12.907Z</v>
       </c>
     </row>
     <row r="33">
@@ -1164,7 +1164,7 @@
         <v/>
       </c>
       <c r="G33" t="str">
-        <v>2026-06-12T09:32:48.571Z</v>
+        <v>2026-06-23T09:24:13.476Z</v>
       </c>
     </row>
     <row r="34">
@@ -1181,13 +1181,13 @@
         <v>PASS</v>
       </c>
       <c r="E34">
-        <v>1105</v>
+        <v>1098</v>
       </c>
       <c r="F34" t="str">
         <v/>
       </c>
       <c r="G34" t="str">
-        <v>2026-06-12T09:32:49.677Z</v>
+        <v>2026-06-23T09:24:14.575Z</v>
       </c>
     </row>
     <row r="35">
@@ -1204,13 +1204,13 @@
         <v>PASS</v>
       </c>
       <c r="E35">
-        <v>689</v>
+        <v>628</v>
       </c>
       <c r="F35" t="str">
         <v/>
       </c>
       <c r="G35" t="str">
-        <v>2026-06-12T09:32:50.368Z</v>
+        <v>2026-06-23T09:24:15.204Z</v>
       </c>
     </row>
     <row r="36">
@@ -1227,13 +1227,13 @@
         <v>PASS</v>
       </c>
       <c r="E36">
-        <v>609</v>
+        <v>634</v>
       </c>
       <c r="F36" t="str">
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>2026-06-12T09:32:50.977Z</v>
+        <v>2026-06-23T09:24:15.838Z</v>
       </c>
     </row>
     <row r="37">
@@ -1250,13 +1250,13 @@
         <v>PASS</v>
       </c>
       <c r="E37">
-        <v>683</v>
+        <v>615</v>
       </c>
       <c r="F37" t="str">
         <v/>
       </c>
       <c r="G37" t="str">
-        <v>2026-06-12T09:32:51.660Z</v>
+        <v>2026-06-23T09:24:16.453Z</v>
       </c>
     </row>
     <row r="38">
@@ -1273,13 +1273,13 @@
         <v>PASS</v>
       </c>
       <c r="E38">
-        <v>599</v>
+        <v>635</v>
       </c>
       <c r="F38" t="str">
         <v/>
       </c>
       <c r="G38" t="str">
-        <v>2026-06-12T09:32:52.259Z</v>
+        <v>2026-06-23T09:24:17.088Z</v>
       </c>
     </row>
     <row r="39">
@@ -1296,13 +1296,13 @@
         <v>PASS</v>
       </c>
       <c r="E39">
-        <v>635</v>
+        <v>615</v>
       </c>
       <c r="F39" t="str">
         <v/>
       </c>
       <c r="G39" t="str">
-        <v>2026-06-12T09:32:52.894Z</v>
+        <v>2026-06-23T09:24:17.703Z</v>
       </c>
     </row>
     <row r="40">
@@ -1319,13 +1319,13 @@
         <v>PASS</v>
       </c>
       <c r="E40">
-        <v>632</v>
+        <v>588</v>
       </c>
       <c r="F40" t="str">
         <v/>
       </c>
       <c r="G40" t="str">
-        <v>2026-06-12T09:32:53.526Z</v>
+        <v>2026-06-23T09:24:18.291Z</v>
       </c>
     </row>
     <row r="41">
@@ -1342,13 +1342,13 @@
         <v>PASS</v>
       </c>
       <c r="E41">
-        <v>643</v>
+        <v>580</v>
       </c>
       <c r="F41" t="str">
         <v/>
       </c>
       <c r="G41" t="str">
-        <v>2026-06-12T09:32:54.169Z</v>
+        <v>2026-06-23T09:24:18.871Z</v>
       </c>
     </row>
     <row r="42">
@@ -1365,13 +1365,13 @@
         <v>PASS</v>
       </c>
       <c r="E42">
-        <v>651</v>
+        <v>600</v>
       </c>
       <c r="F42" t="str">
         <v/>
       </c>
       <c r="G42" t="str">
-        <v>2026-06-12T09:32:54.820Z</v>
+        <v>2026-06-23T09:24:19.471Z</v>
       </c>
     </row>
     <row r="43">
@@ -1388,13 +1388,13 @@
         <v>PASS</v>
       </c>
       <c r="E43">
-        <v>624</v>
+        <v>631</v>
       </c>
       <c r="F43" t="str">
         <v/>
       </c>
       <c r="G43" t="str">
-        <v>2026-06-12T09:32:55.444Z</v>
+        <v>2026-06-23T09:24:20.102Z</v>
       </c>
     </row>
     <row r="44">
@@ -1411,13 +1411,13 @@
         <v>PASS</v>
       </c>
       <c r="E44">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="F44" t="str">
         <v/>
       </c>
       <c r="G44" t="str">
-        <v>2026-06-12T09:32:56.041Z</v>
+        <v>2026-06-23T09:24:20.705Z</v>
       </c>
     </row>
     <row r="45">
@@ -1434,13 +1434,13 @@
         <v>PASS</v>
       </c>
       <c r="E45">
-        <v>634</v>
+        <v>628</v>
       </c>
       <c r="F45" t="str">
         <v/>
       </c>
       <c r="G45" t="str">
-        <v>2026-06-12T09:32:56.675Z</v>
+        <v>2026-06-23T09:24:21.333Z</v>
       </c>
     </row>
     <row r="46">
@@ -1457,13 +1457,13 @@
         <v>PASS</v>
       </c>
       <c r="E46">
-        <v>608</v>
+        <v>619</v>
       </c>
       <c r="F46" t="str">
         <v/>
       </c>
       <c r="G46" t="str">
-        <v>2026-06-12T09:32:57.283Z</v>
+        <v>2026-06-23T09:24:21.952Z</v>
       </c>
     </row>
     <row r="47">
@@ -1480,13 +1480,13 @@
         <v>PASS</v>
       </c>
       <c r="E47">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="F47" t="str">
         <v/>
       </c>
       <c r="G47" t="str">
-        <v>2026-06-12T09:32:57.859Z</v>
+        <v>2026-06-23T09:24:22.525Z</v>
       </c>
     </row>
     <row r="48">
@@ -1503,13 +1503,13 @@
         <v>PASS</v>
       </c>
       <c r="E48">
-        <v>598</v>
+        <v>631</v>
       </c>
       <c r="F48" t="str">
         <v/>
       </c>
       <c r="G48" t="str">
-        <v>2026-06-12T09:32:58.457Z</v>
+        <v>2026-06-23T09:24:23.156Z</v>
       </c>
     </row>
     <row r="49">
@@ -1526,13 +1526,13 @@
         <v>PASS</v>
       </c>
       <c r="E49">
-        <v>636</v>
+        <v>606</v>
       </c>
       <c r="F49" t="str">
         <v/>
       </c>
       <c r="G49" t="str">
-        <v>2026-06-12T09:32:59.093Z</v>
+        <v>2026-06-23T09:24:23.763Z</v>
       </c>
     </row>
     <row r="50">
@@ -1549,13 +1549,13 @@
         <v>PASS</v>
       </c>
       <c r="E50">
-        <v>545</v>
+        <v>525</v>
       </c>
       <c r="F50" t="str">
         <v/>
       </c>
       <c r="G50" t="str">
-        <v>2026-06-12T09:32:59.638Z</v>
+        <v>2026-06-23T09:24:24.288Z</v>
       </c>
     </row>
     <row r="51">
@@ -1572,13 +1572,13 @@
         <v>PASS</v>
       </c>
       <c r="E51">
-        <v>534</v>
+        <v>595</v>
       </c>
       <c r="F51" t="str">
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>2026-06-12T09:33:00.172Z</v>
+        <v>2026-06-23T09:24:24.883Z</v>
       </c>
     </row>
     <row r="52">
@@ -1595,13 +1595,13 @@
         <v>PASS</v>
       </c>
       <c r="E52">
-        <v>371</v>
+        <v>385</v>
       </c>
       <c r="F52" t="str">
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>2026-06-12T09:33:00.544Z</v>
+        <v>2026-06-23T09:24:25.268Z</v>
       </c>
     </row>
     <row r="53">
@@ -1618,13 +1618,13 @@
         <v>PASS</v>
       </c>
       <c r="E53">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="F53" t="str">
         <v/>
       </c>
       <c r="G53" t="str">
-        <v>2026-06-12T09:33:00.569Z</v>
+        <v>2026-06-23T09:24:25.306Z</v>
       </c>
     </row>
     <row r="54">
@@ -1641,13 +1641,13 @@
         <v>PASS</v>
       </c>
       <c r="E54">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F54" t="str">
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>2026-06-12T09:33:00.584Z</v>
+        <v>2026-06-23T09:24:25.319Z</v>
       </c>
     </row>
     <row r="55">
@@ -1664,13 +1664,13 @@
         <v>PASS</v>
       </c>
       <c r="E55">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F55" t="str">
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>2026-06-12T09:33:00.610Z</v>
+        <v>2026-06-23T09:24:25.348Z</v>
       </c>
     </row>
     <row r="56">
@@ -1687,13 +1687,13 @@
         <v>PASS</v>
       </c>
       <c r="E56">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F56" t="str">
         <v/>
       </c>
       <c r="G56" t="str">
-        <v>2026-06-12T09:33:00.638Z</v>
+        <v>2026-06-23T09:24:25.364Z</v>
       </c>
     </row>
     <row r="57">
@@ -1710,13 +1710,13 @@
         <v>PASS</v>
       </c>
       <c r="E57">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F57" t="str">
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>2026-06-12T09:33:00.668Z</v>
+        <v>2026-06-23T09:24:25.376Z</v>
       </c>
     </row>
     <row r="58">
@@ -1733,13 +1733,13 @@
         <v>PASS</v>
       </c>
       <c r="E58">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F58" t="str">
         <v/>
       </c>
       <c r="G58" t="str">
-        <v>2026-06-12T09:33:00.717Z</v>
+        <v>2026-06-23T09:24:25.400Z</v>
       </c>
     </row>
     <row r="59">
@@ -1756,13 +1756,13 @@
         <v>PASS</v>
       </c>
       <c r="E59">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F59" t="str">
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>2026-06-12T09:33:00.733Z</v>
+        <v>2026-06-23T09:24:25.412Z</v>
       </c>
     </row>
     <row r="60">
@@ -1779,13 +1779,13 @@
         <v>PASS</v>
       </c>
       <c r="E60">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F60" t="str">
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>2026-06-12T09:33:00.759Z</v>
+        <v>2026-06-23T09:24:25.435Z</v>
       </c>
     </row>
     <row r="61">
@@ -1802,13 +1802,13 @@
         <v>PASS</v>
       </c>
       <c r="E61">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F61" t="str">
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>2026-06-12T09:33:00.772Z</v>
+        <v>2026-06-23T09:24:25.447Z</v>
       </c>
     </row>
     <row r="62">
@@ -1825,13 +1825,13 @@
         <v>PASS</v>
       </c>
       <c r="E62">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F62" t="str">
         <v/>
       </c>
       <c r="G62" t="str">
-        <v>2026-06-12T09:33:00.783Z</v>
+        <v>2026-06-23T09:24:25.467Z</v>
       </c>
     </row>
     <row r="63">
@@ -1848,13 +1848,13 @@
         <v>PASS</v>
       </c>
       <c r="E63">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F63" t="str">
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.485Z</v>
       </c>
     </row>
     <row r="64">
@@ -1877,7 +1877,7 @@
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.485Z</v>
       </c>
     </row>
     <row r="65">
@@ -1900,7 +1900,7 @@
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.485Z</v>
       </c>
     </row>
     <row r="66">
@@ -1923,7 +1923,7 @@
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.485Z</v>
       </c>
     </row>
     <row r="67">
@@ -1946,7 +1946,7 @@
         <v/>
       </c>
       <c r="G67" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.485Z</v>
       </c>
     </row>
     <row r="68">
@@ -1963,13 +1963,13 @@
         <v>PASS</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F68" t="str">
         <v/>
       </c>
       <c r="G68" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.486Z</v>
       </c>
     </row>
     <row r="69">
@@ -1992,7 +1992,7 @@
         <v/>
       </c>
       <c r="G69" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.486Z</v>
       </c>
     </row>
     <row r="70">
@@ -2015,7 +2015,7 @@
         <v/>
       </c>
       <c r="G70" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.486Z</v>
       </c>
     </row>
     <row r="71">
@@ -2038,7 +2038,7 @@
         <v/>
       </c>
       <c r="G71" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.486Z</v>
       </c>
     </row>
     <row r="72">
@@ -2061,7 +2061,7 @@
         <v/>
       </c>
       <c r="G72" t="str">
-        <v>2026-06-12T09:33:00.810Z</v>
+        <v>2026-06-23T09:24:25.486Z</v>
       </c>
     </row>
     <row r="73">
@@ -2078,13 +2078,13 @@
         <v>PASS</v>
       </c>
       <c r="E73">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F73" t="str">
         <v/>
       </c>
       <c r="G73" t="str">
-        <v>2026-06-12T09:33:00.831Z</v>
+        <v>2026-06-23T09:24:25.506Z</v>
       </c>
     </row>
     <row r="74">
@@ -2101,13 +2101,13 @@
         <v>PASS</v>
       </c>
       <c r="E74">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="F74" t="str">
         <v/>
       </c>
       <c r="G74" t="str">
-        <v>2026-06-12T09:33:00.921Z</v>
+        <v>2026-06-23T09:24:25.622Z</v>
       </c>
     </row>
     <row r="75">
@@ -2124,13 +2124,13 @@
         <v>PASS</v>
       </c>
       <c r="E75">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="F75" t="str">
         <v/>
       </c>
       <c r="G75" t="str">
-        <v>2026-06-12T09:33:00.990Z</v>
+        <v>2026-06-23T09:24:25.652Z</v>
       </c>
     </row>
     <row r="76">
@@ -2147,13 +2147,13 @@
         <v>PASS</v>
       </c>
       <c r="E76">
-        <v>35</v>
+        <v>112</v>
       </c>
       <c r="F76" t="str">
         <v/>
       </c>
       <c r="G76" t="str">
-        <v>2026-06-12T09:33:01.025Z</v>
+        <v>2026-06-23T09:24:25.764Z</v>
       </c>
     </row>
     <row r="77">
@@ -2170,13 +2170,13 @@
         <v>PASS</v>
       </c>
       <c r="E77">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F77" t="str">
         <v/>
       </c>
       <c r="G77" t="str">
-        <v>2026-06-12T09:33:01.037Z</v>
+        <v>2026-06-23T09:24:25.778Z</v>
       </c>
     </row>
     <row r="78">
@@ -2193,13 +2193,13 @@
         <v>PASS</v>
       </c>
       <c r="E78">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F78" t="str">
         <v/>
       </c>
       <c r="G78" t="str">
-        <v>2026-06-12T09:33:01.051Z</v>
+        <v>2026-06-23T09:24:25.793Z</v>
       </c>
     </row>
     <row r="79">
@@ -2216,13 +2216,13 @@
         <v>PASS</v>
       </c>
       <c r="E79">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F79" t="str">
         <v/>
       </c>
       <c r="G79" t="str">
-        <v>2026-06-12T09:33:01.059Z</v>
+        <v>2026-06-23T09:24:25.802Z</v>
       </c>
     </row>
     <row r="80">
@@ -2245,7 +2245,7 @@
         <v/>
       </c>
       <c r="G80" t="str">
-        <v>2026-06-12T09:33:01.075Z</v>
+        <v>2026-06-23T09:24:25.818Z</v>
       </c>
     </row>
     <row r="81">
@@ -2262,13 +2262,13 @@
         <v>PASS</v>
       </c>
       <c r="E81">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="F81" t="str">
         <v/>
       </c>
       <c r="G81" t="str">
-        <v>2026-06-12T09:33:02.445Z</v>
+        <v>2026-06-23T09:24:27.186Z</v>
       </c>
     </row>
     <row r="82">
@@ -2285,13 +2285,13 @@
         <v>PASS</v>
       </c>
       <c r="E82">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F82" t="str">
         <v/>
       </c>
       <c r="G82" t="str">
-        <v>2026-06-12T09:33:02.475Z</v>
+        <v>2026-06-23T09:24:27.205Z</v>
       </c>
     </row>
     <row r="83">
@@ -2308,13 +2308,13 @@
         <v>PASS</v>
       </c>
       <c r="E83">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="F83" t="str">
         <v/>
       </c>
       <c r="G83" t="str">
-        <v>2026-06-12T09:33:03.535Z</v>
+        <v>2026-06-23T09:24:28.263Z</v>
       </c>
     </row>
     <row r="84">
@@ -2331,13 +2331,13 @@
         <v>PASS</v>
       </c>
       <c r="E84">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F84" t="str">
         <v/>
       </c>
       <c r="G84" t="str">
-        <v>2026-06-12T09:33:03.553Z</v>
+        <v>2026-06-23T09:24:28.278Z</v>
       </c>
     </row>
     <row r="85">
@@ -2354,13 +2354,13 @@
         <v>PASS</v>
       </c>
       <c r="E85">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F85" t="str">
         <v/>
       </c>
       <c r="G85" t="str">
-        <v>2026-06-12T09:33:03.569Z</v>
+        <v>2026-06-23T09:24:28.287Z</v>
       </c>
     </row>
     <row r="86">
@@ -2377,13 +2377,13 @@
         <v>PASS</v>
       </c>
       <c r="E86">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F86" t="str">
         <v/>
       </c>
       <c r="G86" t="str">
-        <v>2026-06-12T09:33:03.578Z</v>
+        <v>2026-06-23T09:24:28.294Z</v>
       </c>
     </row>
     <row r="87">
@@ -2400,13 +2400,13 @@
         <v>PASS</v>
       </c>
       <c r="E87">
-        <v>1044</v>
+        <v>1019</v>
       </c>
       <c r="F87" t="str">
         <v/>
       </c>
       <c r="G87" t="str">
-        <v>2026-06-12T09:33:04.623Z</v>
+        <v>2026-06-23T09:24:29.313Z</v>
       </c>
     </row>
     <row r="88">
@@ -2423,13 +2423,13 @@
         <v>PASS</v>
       </c>
       <c r="E88">
-        <v>1089</v>
+        <v>1073</v>
       </c>
       <c r="F88" t="str">
         <v/>
       </c>
       <c r="G88" t="str">
-        <v>2026-06-12T09:33:05.713Z</v>
+        <v>2026-06-23T09:24:30.386Z</v>
       </c>
     </row>
     <row r="89">
@@ -2446,13 +2446,13 @@
         <v>PASS</v>
       </c>
       <c r="E89">
-        <v>1186</v>
+        <v>1226</v>
       </c>
       <c r="F89" t="str">
         <v/>
       </c>
       <c r="G89" t="str">
-        <v>2026-06-12T09:33:06.900Z</v>
+        <v>2026-06-23T09:24:31.612Z</v>
       </c>
     </row>
     <row r="90">
@@ -2469,13 +2469,13 @@
         <v>PASS</v>
       </c>
       <c r="E90">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F90" t="str">
         <v/>
       </c>
       <c r="G90" t="str">
-        <v>2026-06-12T09:33:06.937Z</v>
+        <v>2026-06-23T09:24:31.633Z</v>
       </c>
     </row>
     <row r="91">
@@ -2492,13 +2492,13 @@
         <v>PASS</v>
       </c>
       <c r="E91">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="F91" t="str">
         <v/>
       </c>
       <c r="G91" t="str">
-        <v>2026-06-12T09:33:07.778Z</v>
+        <v>2026-06-23T09:24:32.470Z</v>
       </c>
     </row>
     <row r="92">
@@ -2521,7 +2521,7 @@
         <v/>
       </c>
       <c r="G92" t="str">
-        <v>2026-06-12T09:33:08.618Z</v>
+        <v>2026-06-23T09:24:33.310Z</v>
       </c>
     </row>
     <row r="93">
@@ -2538,13 +2538,13 @@
         <v>PASS</v>
       </c>
       <c r="E93">
-        <v>961</v>
+        <v>978</v>
       </c>
       <c r="F93" t="str">
         <v/>
       </c>
       <c r="G93" t="str">
-        <v>2026-06-12T09:33:09.579Z</v>
+        <v>2026-06-23T09:24:34.288Z</v>
       </c>
     </row>
     <row r="94">
@@ -2561,13 +2561,13 @@
         <v>PASS</v>
       </c>
       <c r="E94">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F94" t="str">
         <v/>
       </c>
       <c r="G94" t="str">
-        <v>2026-06-12T09:33:09.610Z</v>
+        <v>2026-06-23T09:24:34.310Z</v>
       </c>
     </row>
     <row r="95">
@@ -2584,13 +2584,13 @@
         <v>PASS</v>
       </c>
       <c r="E95">
-        <v>193</v>
+        <v>134</v>
       </c>
       <c r="F95" t="str">
         <v/>
       </c>
       <c r="G95" t="str">
-        <v>2026-06-12T09:33:09.803Z</v>
+        <v>2026-06-23T09:24:34.445Z</v>
       </c>
     </row>
     <row r="96">
@@ -2607,13 +2607,13 @@
         <v>PASS</v>
       </c>
       <c r="E96">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F96" t="str">
         <v/>
       </c>
       <c r="G96" t="str">
-        <v>2026-06-12T09:33:09.905Z</v>
+        <v>2026-06-23T09:24:34.540Z</v>
       </c>
     </row>
     <row r="97">
@@ -2630,13 +2630,13 @@
         <v>PASS</v>
       </c>
       <c r="E97">
-        <v>2253</v>
+        <v>2192</v>
       </c>
       <c r="F97" t="str">
         <v/>
       </c>
       <c r="G97" t="str">
-        <v>2026-06-12T09:33:12.158Z</v>
+        <v>2026-06-23T09:24:36.732Z</v>
       </c>
     </row>
     <row r="98">
@@ -2653,13 +2653,13 @@
         <v>PASS</v>
       </c>
       <c r="E98">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="F98" t="str">
         <v/>
       </c>
       <c r="G98" t="str">
-        <v>2026-06-12T09:33:12.242Z</v>
+        <v>2026-06-23T09:24:36.826Z</v>
       </c>
     </row>
     <row r="99">
@@ -2676,13 +2676,13 @@
         <v>PASS</v>
       </c>
       <c r="E99">
-        <v>1746</v>
+        <v>1735</v>
       </c>
       <c r="F99" t="str">
         <v/>
       </c>
       <c r="G99" t="str">
-        <v>2026-06-12T09:33:13.988Z</v>
+        <v>2026-06-23T09:24:38.561Z</v>
       </c>
     </row>
     <row r="100">
@@ -2699,13 +2699,13 @@
         <v>PASS</v>
       </c>
       <c r="E100">
-        <v>91</v>
+        <v>45</v>
       </c>
       <c r="F100" t="str">
         <v/>
       </c>
       <c r="G100" t="str">
-        <v>2026-06-12T09:33:14.079Z</v>
+        <v>2026-06-23T09:24:38.607Z</v>
       </c>
     </row>
     <row r="101">
@@ -2722,13 +2722,13 @@
         <v>PASS</v>
       </c>
       <c r="E101">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="F101" t="str">
         <v/>
       </c>
       <c r="G101" t="str">
-        <v>2026-06-12T09:33:14.154Z</v>
+        <v>2026-06-23T09:24:38.650Z</v>
       </c>
     </row>
     <row r="102">
@@ -2745,13 +2745,13 @@
         <v>PASS</v>
       </c>
       <c r="E102">
-        <v>1584</v>
+        <v>1535</v>
       </c>
       <c r="F102" t="str">
         <v/>
       </c>
       <c r="G102" t="str">
-        <v>2026-06-12T09:33:15.738Z</v>
+        <v>2026-06-23T09:24:40.185Z</v>
       </c>
     </row>
     <row r="103">
@@ -2768,13 +2768,13 @@
         <v>PASS</v>
       </c>
       <c r="E103">
-        <v>122</v>
+        <v>67</v>
       </c>
       <c r="F103" t="str">
         <v/>
       </c>
       <c r="G103" t="str">
-        <v>2026-06-12T09:33:15.860Z</v>
+        <v>2026-06-23T09:24:40.252Z</v>
       </c>
     </row>
     <row r="104">
@@ -2791,13 +2791,13 @@
         <v>PASS</v>
       </c>
       <c r="E104">
-        <v>896</v>
+        <v>880</v>
       </c>
       <c r="F104" t="str">
         <v/>
       </c>
       <c r="G104" t="str">
-        <v>2026-06-12T09:33:16.756Z</v>
+        <v>2026-06-23T09:24:41.132Z</v>
       </c>
     </row>
     <row r="105">
@@ -2814,13 +2814,13 @@
         <v>PASS</v>
       </c>
       <c r="E105">
-        <v>130</v>
+        <v>56</v>
       </c>
       <c r="F105" t="str">
         <v/>
       </c>
       <c r="G105" t="str">
-        <v>2026-06-12T09:33:16.886Z</v>
+        <v>2026-06-23T09:24:41.188Z</v>
       </c>
     </row>
     <row r="106">
@@ -2837,13 +2837,13 @@
         <v>PASS</v>
       </c>
       <c r="E106">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="F106" t="str">
         <v/>
       </c>
       <c r="G106" t="str">
-        <v>2026-06-12T09:33:16.955Z</v>
+        <v>2026-06-23T09:24:41.204Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>